<commit_message>
Fix: add ChemDoodle to root index.html
</commit_message>
<xml_diff>
--- a/Concours_Blanc_1.xlsx
+++ b/Concours_Blanc_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOULAY\Desktop\WEB_TEST_APP\MED-CONTEST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{886BE765-35F0-42A0-8B63-8D2ADAE84808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0108D6FF-577A-4BE9-9D3A-77869DCE9F43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="513">
   <si>
     <t>Option 1</t>
   </si>
@@ -384,9 +384,6 @@
   </si>
   <si>
     <t>(E) : $a&gt;0$ et $b=0$</t>
-  </si>
-  <si>
-    <t>MEDECINE 2020</t>
   </si>
   <si>
     <t>CHIMIE</t>
@@ -1658,6 +1655,9 @@
   </si>
   <si>
     <t>Numéro de concours</t>
+  </si>
+  <si>
+    <t>Concours Blanc 1</t>
   </si>
 </sst>
 </file>
@@ -1722,7 +1722,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1747,9 +1747,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2086,8 +2083,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
-        <v>512</v>
+      <c r="A1" s="12" t="s">
+        <v>511</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>14</v>
@@ -2127,754 +2124,794 @@
       </c>
     </row>
     <row r="2" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="14">
+      <c r="A2" s="13">
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="12" t="s">
-        <v>331</v>
+      <c r="C2" s="11" t="s">
+        <v>330</v>
       </c>
       <c r="D2" s="2"/>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="F2" s="11" t="s">
         <v>231</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="G2" s="11" t="s">
         <v>232</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="H2" s="11" t="s">
         <v>233</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="I2" s="11" t="s">
         <v>234</v>
       </c>
-      <c r="I2" s="12" t="s">
-        <v>235</v>
-      </c>
-      <c r="J2" s="12" t="s">
-        <v>235</v>
+      <c r="J2" s="11" t="s">
+        <v>234</v>
       </c>
       <c r="K2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="5"/>
+      <c r="L2" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M2" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="14">
+      <c r="A3" s="13">
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="12" t="s">
-        <v>332</v>
+      <c r="C3" s="11" t="s">
+        <v>331</v>
       </c>
       <c r="D3" s="2"/>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="F3" s="11" t="s">
         <v>236</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="G3" s="11" t="s">
         <v>237</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="H3" s="11" t="s">
         <v>238</v>
       </c>
-      <c r="H3" s="12" t="s">
+      <c r="I3" s="11" t="s">
         <v>239</v>
       </c>
-      <c r="I3" s="12" t="s">
-        <v>240</v>
-      </c>
-      <c r="J3" s="12" t="s">
-        <v>238</v>
+      <c r="J3" s="11" t="s">
+        <v>237</v>
       </c>
       <c r="K3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L3" s="5"/>
+      <c r="L3" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M3" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="75" x14ac:dyDescent="0.25">
-      <c r="A4" s="14">
+      <c r="A4" s="13">
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="12" t="s">
-        <v>333</v>
+      <c r="C4" s="11" t="s">
+        <v>332</v>
       </c>
       <c r="D4" s="2"/>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="F4" s="11" t="s">
         <v>241</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="G4" s="11" t="s">
         <v>242</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="11" t="s">
         <v>243</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="I4" s="11" t="s">
         <v>244</v>
       </c>
-      <c r="I4" s="12" t="s">
-        <v>245</v>
-      </c>
-      <c r="J4" s="12" t="s">
-        <v>242</v>
+      <c r="J4" s="11" t="s">
+        <v>241</v>
       </c>
       <c r="K4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L4" s="5"/>
+      <c r="L4" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M4" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="14">
+      <c r="A5" s="13">
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="12" t="s">
-        <v>334</v>
+      <c r="C5" s="11" t="s">
+        <v>333</v>
       </c>
       <c r="D5" s="2"/>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="F5" s="11" t="s">
         <v>246</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="G5" s="11" t="s">
         <v>247</v>
       </c>
-      <c r="G5" s="12" t="s">
+      <c r="H5" s="11" t="s">
         <v>248</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="I5" s="11" t="s">
         <v>249</v>
       </c>
-      <c r="I5" s="12" t="s">
-        <v>250</v>
-      </c>
-      <c r="J5" s="12" t="s">
-        <v>246</v>
+      <c r="J5" s="11" t="s">
+        <v>245</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="5"/>
+      <c r="L5" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M5" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="75" x14ac:dyDescent="0.25">
-      <c r="A6" s="14">
+      <c r="A6" s="13">
         <v>1</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="12" t="s">
-        <v>335</v>
+      <c r="C6" s="11" t="s">
+        <v>334</v>
       </c>
       <c r="D6" s="2"/>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="F6" s="11" t="s">
         <v>251</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="G6" s="11" t="s">
         <v>252</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="H6" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="H6" s="12" t="s">
+      <c r="I6" s="11" t="s">
         <v>254</v>
       </c>
-      <c r="I6" s="12" t="s">
-        <v>255</v>
-      </c>
-      <c r="J6" s="12" t="s">
-        <v>255</v>
+      <c r="J6" s="11" t="s">
+        <v>254</v>
       </c>
       <c r="K6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="5"/>
+      <c r="L6" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M6" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="14">
+      <c r="A7" s="13">
         <v>1</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="12" t="s">
-        <v>336</v>
+      <c r="C7" s="11" t="s">
+        <v>335</v>
       </c>
       <c r="D7" s="2"/>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="11" t="s">
+        <v>255</v>
+      </c>
+      <c r="F7" s="11" t="s">
         <v>256</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="G7" s="11" t="s">
         <v>257</v>
       </c>
-      <c r="G7" s="12" t="s">
+      <c r="H7" s="11" t="s">
         <v>258</v>
       </c>
-      <c r="H7" s="12" t="s">
+      <c r="I7" s="11" t="s">
         <v>259</v>
       </c>
-      <c r="I7" s="12" t="s">
-        <v>260</v>
-      </c>
-      <c r="J7" s="12" t="s">
-        <v>258</v>
+      <c r="J7" s="11" t="s">
+        <v>257</v>
       </c>
       <c r="K7" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L7" s="5"/>
+      <c r="L7" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M7" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="120" x14ac:dyDescent="0.25">
-      <c r="A8" s="14">
+      <c r="A8" s="13">
         <v>1</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="12" t="s">
-        <v>337</v>
+      <c r="C8" s="11" t="s">
+        <v>336</v>
       </c>
       <c r="D8" s="2"/>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="F8" s="11" t="s">
         <v>261</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="G8" s="11" t="s">
         <v>262</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="H8" s="11" t="s">
         <v>263</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="I8" s="11" t="s">
         <v>264</v>
       </c>
-      <c r="I8" s="12" t="s">
-        <v>265</v>
-      </c>
-      <c r="J8" s="12" t="s">
-        <v>265</v>
+      <c r="J8" s="11" t="s">
+        <v>264</v>
       </c>
       <c r="K8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L8" s="5"/>
+      <c r="L8" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M8" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="14">
+      <c r="A9" s="13">
         <v>1</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="12" t="s">
-        <v>338</v>
+      <c r="C9" s="11" t="s">
+        <v>337</v>
       </c>
       <c r="D9" s="2"/>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="F9" s="11" t="s">
         <v>266</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="G9" s="11" t="s">
         <v>267</v>
       </c>
-      <c r="G9" s="12" t="s">
+      <c r="H9" s="11" t="s">
         <v>268</v>
       </c>
-      <c r="H9" s="12" t="s">
+      <c r="I9" s="11" t="s">
         <v>269</v>
       </c>
-      <c r="I9" s="12" t="s">
-        <v>270</v>
-      </c>
-      <c r="J9" s="12" t="s">
-        <v>270</v>
+      <c r="J9" s="11" t="s">
+        <v>269</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L9" s="5"/>
+      <c r="L9" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M9" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="14">
+      <c r="A10" s="13">
         <v>1</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="12" t="s">
-        <v>339</v>
+      <c r="C10" s="11" t="s">
+        <v>338</v>
       </c>
       <c r="D10" s="2"/>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="11" t="s">
+        <v>270</v>
+      </c>
+      <c r="F10" s="11" t="s">
         <v>271</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="G10" s="11" t="s">
         <v>272</v>
       </c>
-      <c r="G10" s="12" t="s">
+      <c r="H10" s="11" t="s">
         <v>273</v>
       </c>
-      <c r="H10" s="12" t="s">
+      <c r="I10" s="11" t="s">
         <v>274</v>
       </c>
-      <c r="I10" s="12" t="s">
-        <v>275</v>
-      </c>
-      <c r="J10" s="12" t="s">
-        <v>271</v>
+      <c r="J10" s="11" t="s">
+        <v>270</v>
       </c>
       <c r="K10" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L10" s="5"/>
+      <c r="L10" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M10" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="14">
+      <c r="A11" s="13">
         <v>1</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="12" t="s">
-        <v>340</v>
+      <c r="C11" s="11" t="s">
+        <v>339</v>
       </c>
       <c r="D11" s="2"/>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="F11" s="11" t="s">
         <v>276</v>
       </c>
-      <c r="F11" s="12" t="s">
+      <c r="G11" s="11" t="s">
         <v>277</v>
       </c>
-      <c r="G11" s="12" t="s">
+      <c r="H11" s="11" t="s">
         <v>278</v>
       </c>
-      <c r="H11" s="12" t="s">
+      <c r="I11" s="11" t="s">
         <v>279</v>
       </c>
-      <c r="I11" s="12" t="s">
-        <v>280</v>
-      </c>
-      <c r="J11" s="12" t="s">
-        <v>280</v>
+      <c r="J11" s="11" t="s">
+        <v>279</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L11" s="5"/>
+      <c r="L11" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M11" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="345" x14ac:dyDescent="0.25">
-      <c r="A12" s="14">
+      <c r="A12" s="13">
         <v>1</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>464</v>
+      <c r="C12" s="11" t="s">
+        <v>463</v>
       </c>
       <c r="D12" s="2"/>
-      <c r="E12" s="12" t="s">
+      <c r="E12" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="F12" s="11" t="s">
         <v>281</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="G12" s="11" t="s">
         <v>282</v>
       </c>
-      <c r="G12" s="12" t="s">
+      <c r="H12" s="11" t="s">
         <v>283</v>
       </c>
-      <c r="H12" s="12" t="s">
+      <c r="I12" s="11" t="s">
         <v>284</v>
       </c>
-      <c r="I12" s="12" t="s">
-        <v>285</v>
-      </c>
-      <c r="J12" s="12" t="s">
-        <v>283</v>
+      <c r="J12" s="11" t="s">
+        <v>282</v>
       </c>
       <c r="K12" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L12" s="5"/>
+      <c r="L12" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M12" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="90" x14ac:dyDescent="0.25">
-      <c r="A13" s="14">
+      <c r="A13" s="13">
         <v>1</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="12" t="s">
-        <v>458</v>
+      <c r="C13" s="11" t="s">
+        <v>457</v>
       </c>
       <c r="D13" s="2"/>
-      <c r="E13" s="12" t="s">
+      <c r="E13" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="F13" s="11" t="s">
         <v>286</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="G13" s="11" t="s">
         <v>287</v>
       </c>
-      <c r="G13" s="12" t="s">
+      <c r="H13" s="11" t="s">
         <v>288</v>
       </c>
-      <c r="H13" s="12" t="s">
+      <c r="I13" s="11" t="s">
         <v>289</v>
       </c>
-      <c r="I13" s="12" t="s">
-        <v>290</v>
-      </c>
-      <c r="J13" s="12" t="s">
-        <v>289</v>
+      <c r="J13" s="11" t="s">
+        <v>288</v>
       </c>
       <c r="K13" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L13" s="5"/>
+      <c r="L13" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M13" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="105" x14ac:dyDescent="0.25">
-      <c r="A14" s="14">
+      <c r="A14" s="13">
         <v>1</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="12" t="s">
-        <v>459</v>
+      <c r="C14" s="11" t="s">
+        <v>458</v>
       </c>
       <c r="D14" s="2"/>
-      <c r="E14" s="12" t="s">
+      <c r="E14" s="11" t="s">
+        <v>290</v>
+      </c>
+      <c r="F14" s="11" t="s">
         <v>291</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="G14" s="11" t="s">
         <v>292</v>
       </c>
-      <c r="G14" s="12" t="s">
+      <c r="H14" s="11" t="s">
         <v>293</v>
       </c>
-      <c r="H14" s="12" t="s">
+      <c r="I14" s="11" t="s">
         <v>294</v>
       </c>
-      <c r="I14" s="12" t="s">
-        <v>295</v>
-      </c>
-      <c r="J14" s="12" t="s">
-        <v>291</v>
+      <c r="J14" s="11" t="s">
+        <v>290</v>
       </c>
       <c r="K14" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L14" s="5"/>
+      <c r="L14" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M14" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="14">
+      <c r="A15" s="13">
         <v>1</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="12" t="s">
-        <v>341</v>
+      <c r="C15" s="11" t="s">
+        <v>340</v>
       </c>
       <c r="D15" s="2"/>
-      <c r="E15" s="12" t="s">
+      <c r="E15" s="11" t="s">
+        <v>295</v>
+      </c>
+      <c r="F15" s="11" t="s">
         <v>296</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="G15" s="11" t="s">
         <v>297</v>
       </c>
-      <c r="G15" s="12" t="s">
+      <c r="H15" s="11" t="s">
         <v>298</v>
       </c>
-      <c r="H15" s="12" t="s">
+      <c r="I15" s="11" t="s">
         <v>299</v>
       </c>
-      <c r="I15" s="12" t="s">
-        <v>300</v>
-      </c>
-      <c r="J15" s="12" t="s">
-        <v>299</v>
+      <c r="J15" s="11" t="s">
+        <v>298</v>
       </c>
       <c r="K15" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L15" s="5"/>
+      <c r="L15" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M15" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="105" x14ac:dyDescent="0.25">
-      <c r="A16" s="14">
+      <c r="A16" s="13">
         <v>1</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="12" t="s">
-        <v>460</v>
+      <c r="C16" s="11" t="s">
+        <v>459</v>
       </c>
       <c r="D16" s="2"/>
-      <c r="E16" s="12" t="s">
+      <c r="E16" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="F16" s="11" t="s">
         <v>301</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="G16" s="11" t="s">
         <v>302</v>
       </c>
-      <c r="G16" s="12" t="s">
+      <c r="H16" s="11" t="s">
         <v>303</v>
       </c>
-      <c r="H16" s="12" t="s">
+      <c r="I16" s="11" t="s">
         <v>304</v>
       </c>
-      <c r="I16" s="12" t="s">
-        <v>305</v>
-      </c>
-      <c r="J16" s="12" t="s">
-        <v>301</v>
+      <c r="J16" s="11" t="s">
+        <v>300</v>
       </c>
       <c r="K16" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L16" s="5"/>
+      <c r="L16" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M16" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="75" x14ac:dyDescent="0.25">
-      <c r="A17" s="14">
+      <c r="A17" s="13">
         <v>1</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="12" t="s">
-        <v>342</v>
+      <c r="C17" s="11" t="s">
+        <v>341</v>
       </c>
       <c r="D17" s="2"/>
-      <c r="E17" s="12" t="s">
+      <c r="E17" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="F17" s="11" t="s">
         <v>306</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="G17" s="11" t="s">
         <v>307</v>
       </c>
-      <c r="G17" s="12" t="s">
+      <c r="H17" s="11" t="s">
         <v>308</v>
       </c>
-      <c r="H17" s="12" t="s">
+      <c r="I17" s="11" t="s">
         <v>309</v>
       </c>
-      <c r="I17" s="12" t="s">
-        <v>310</v>
-      </c>
-      <c r="J17" s="12" t="s">
-        <v>310</v>
+      <c r="J17" s="11" t="s">
+        <v>309</v>
       </c>
       <c r="K17" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L17" s="5"/>
+      <c r="L17" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M17" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="135" x14ac:dyDescent="0.25">
-      <c r="A18" s="14">
+      <c r="A18" s="13">
         <v>1</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="12" t="s">
-        <v>461</v>
+      <c r="C18" s="11" t="s">
+        <v>460</v>
       </c>
       <c r="D18" s="2"/>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="11" t="s">
+        <v>310</v>
+      </c>
+      <c r="F18" s="11" t="s">
         <v>311</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="G18" s="11" t="s">
         <v>312</v>
       </c>
-      <c r="G18" s="12" t="s">
+      <c r="H18" s="11" t="s">
         <v>313</v>
       </c>
-      <c r="H18" s="12" t="s">
+      <c r="I18" s="11" t="s">
         <v>314</v>
       </c>
-      <c r="I18" s="12" t="s">
-        <v>315</v>
-      </c>
-      <c r="J18" s="12" t="s">
-        <v>313</v>
+      <c r="J18" s="11" t="s">
+        <v>312</v>
       </c>
       <c r="K18" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L18" s="5"/>
+      <c r="L18" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M18" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="120" x14ac:dyDescent="0.25">
-      <c r="A19" s="14">
+      <c r="A19" s="13">
         <v>1</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C19" s="12" t="s">
-        <v>462</v>
+      <c r="C19" s="11" t="s">
+        <v>461</v>
       </c>
       <c r="D19" s="2"/>
-      <c r="E19" s="12" t="s">
+      <c r="E19" s="11" t="s">
+        <v>315</v>
+      </c>
+      <c r="F19" s="11" t="s">
         <v>316</v>
       </c>
-      <c r="F19" s="12" t="s">
+      <c r="G19" s="11" t="s">
         <v>317</v>
       </c>
-      <c r="G19" s="12" t="s">
+      <c r="H19" s="11" t="s">
         <v>318</v>
       </c>
-      <c r="H19" s="12" t="s">
+      <c r="I19" s="11" t="s">
         <v>319</v>
       </c>
-      <c r="I19" s="12" t="s">
-        <v>320</v>
-      </c>
-      <c r="J19" s="12" t="s">
-        <v>316</v>
+      <c r="J19" s="11" t="s">
+        <v>315</v>
       </c>
       <c r="K19" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L19" s="5"/>
+      <c r="L19" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M19" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="180" x14ac:dyDescent="0.25">
-      <c r="A20" s="14">
+      <c r="A20" s="13">
         <v>1</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="12" t="s">
-        <v>457</v>
+      <c r="C20" s="11" t="s">
+        <v>456</v>
       </c>
       <c r="D20" s="2"/>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="11" t="s">
+        <v>320</v>
+      </c>
+      <c r="F20" s="11" t="s">
         <v>321</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="G20" s="11" t="s">
         <v>322</v>
       </c>
-      <c r="G20" s="12" t="s">
+      <c r="H20" s="11" t="s">
         <v>323</v>
       </c>
-      <c r="H20" s="12" t="s">
+      <c r="I20" s="11" t="s">
         <v>324</v>
       </c>
-      <c r="I20" s="12" t="s">
-        <v>325</v>
-      </c>
-      <c r="J20" s="12" t="s">
-        <v>321</v>
+      <c r="J20" s="11" t="s">
+        <v>320</v>
       </c>
       <c r="K20" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L20" s="5"/>
+      <c r="L20" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M20" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="75" x14ac:dyDescent="0.25">
-      <c r="A21" s="14">
+      <c r="A21" s="13">
         <v>1</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C21" s="12" t="s">
-        <v>463</v>
+      <c r="C21" s="11" t="s">
+        <v>462</v>
       </c>
       <c r="D21" s="2"/>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="11" t="s">
+        <v>325</v>
+      </c>
+      <c r="F21" s="11" t="s">
         <v>326</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="G21" s="11" t="s">
         <v>327</v>
       </c>
-      <c r="G21" s="12" t="s">
+      <c r="H21" s="11" t="s">
         <v>328</v>
       </c>
-      <c r="H21" s="12" t="s">
+      <c r="I21" s="11" t="s">
         <v>329</v>
       </c>
-      <c r="I21" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="J21" s="12" t="s">
-        <v>330</v>
+      <c r="J21" s="11" t="s">
+        <v>329</v>
       </c>
       <c r="K21" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L21" s="5"/>
+      <c r="L21" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M21" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="165" x14ac:dyDescent="0.25">
-      <c r="A22" s="14">
+      <c r="A22" s="13">
         <v>1</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="2"/>
@@ -2886,123 +2923,131 @@
       <c r="K22" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="L22" s="5"/>
+      <c r="L22" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M22" s="5"/>
     </row>
     <row r="23" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="14">
+      <c r="A23" s="13">
         <v>1</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="3" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F23" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="G23" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="H23" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="H23" s="3" t="s">
+      <c r="I23" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="I23" s="3" t="s">
-        <v>121</v>
-      </c>
       <c r="J23" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
+      <c r="L23" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M23" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="14">
+      <c r="A24" s="13">
         <v>1</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="F24" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="G24" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="G24" s="3" t="s">
+      <c r="H24" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="H24" s="3" t="s">
+      <c r="I24" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="I24" s="3" t="s">
-        <v>126</v>
-      </c>
       <c r="J24" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K24" s="5"/>
-      <c r="L24" s="5"/>
+      <c r="L24" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M24" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="14">
+      <c r="A25" s="13">
         <v>1</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="F25" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="G25" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="G25" s="3" t="s">
+      <c r="H25" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="H25" s="3" t="s">
+      <c r="I25" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="I25" s="3" t="s">
-        <v>131</v>
-      </c>
       <c r="J25" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K25" s="5"/>
-      <c r="L25" s="5"/>
+      <c r="L25" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M25" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="105" x14ac:dyDescent="0.25">
-      <c r="A26" s="14">
+      <c r="A26" s="13">
         <v>1</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -3015,89 +3060,93 @@
         <v>9</v>
       </c>
       <c r="L26" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M26" s="5"/>
     </row>
     <row r="27" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="14">
+      <c r="A27" s="13">
         <v>1</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="F27" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="G27" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="H27" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="H27" s="3" t="s">
+      <c r="I27" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="I27" s="3" t="s">
-        <v>136</v>
-      </c>
       <c r="J27" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K27" s="5"/>
-      <c r="L27" s="5"/>
+      <c r="L27" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M27" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A28" s="14">
+      <c r="A28" s="13">
         <v>1</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="F28" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="G28" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="G28" s="3" t="s">
+      <c r="H28" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="H28" s="3" t="s">
+      <c r="I28" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="I28" s="3" t="s">
-        <v>141</v>
-      </c>
       <c r="J28" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K28" s="5"/>
-      <c r="L28" s="5"/>
+      <c r="L28" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M28" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="210" x14ac:dyDescent="0.25">
-      <c r="A29" s="14">
+      <c r="A29" s="13">
         <v>1</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
@@ -3110,124 +3159,130 @@
         <v>9</v>
       </c>
       <c r="L29" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M29" s="5"/>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A30" s="14">
+      <c r="A30" s="13">
         <v>1</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="G30" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="H30" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="I30" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="I30" s="2" t="s">
-        <v>146</v>
-      </c>
       <c r="J30" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="K30" s="5"/>
-      <c r="L30" s="5"/>
+      <c r="L30" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M30" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="14">
+      <c r="A31" s="13">
         <v>1</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="G31" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="G31" s="2" t="s">
+      <c r="H31" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="H31" s="2" t="s">
-        <v>150</v>
-      </c>
       <c r="I31" s="3" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="K31" s="5"/>
-      <c r="L31" s="5"/>
+      <c r="L31" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M31" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:13" ht="135" x14ac:dyDescent="0.25">
-      <c r="A32" s="14">
+      <c r="A32" s="13">
         <v>1</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="F32" s="2" t="s">
+      <c r="G32" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="H32" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="I32" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="I32" s="2" t="s">
-        <v>155</v>
-      </c>
       <c r="J32" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K32" s="5"/>
-      <c r="L32" s="5"/>
+      <c r="L32" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M32" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:13" ht="165" x14ac:dyDescent="0.25">
-      <c r="A33" s="14">
+      <c r="A33" s="13">
         <v>1</v>
       </c>
       <c r="B33" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
@@ -3240,89 +3295,93 @@
         <v>9</v>
       </c>
       <c r="L33" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M33" s="5"/>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A34" s="14">
+      <c r="A34" s="13">
         <v>1</v>
       </c>
       <c r="B34" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="G34" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="H34" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="H34" s="2" t="s">
+      <c r="I34" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I34" s="2" t="s">
-        <v>160</v>
-      </c>
       <c r="J34" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K34" s="5"/>
-      <c r="L34" s="5"/>
+      <c r="L34" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M34" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A35" s="14">
+      <c r="A35" s="13">
         <v>1</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="F35" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="G35" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="H35" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="H35" s="2" t="s">
+      <c r="I35" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="I35" s="2" t="s">
-        <v>165</v>
-      </c>
       <c r="J35" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K35" s="5"/>
-      <c r="L35" s="5"/>
+      <c r="L35" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M35" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:13" ht="240" x14ac:dyDescent="0.25">
-      <c r="A36" s="14">
+      <c r="A36" s="13">
         <v>1</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
@@ -3335,89 +3394,93 @@
         <v>9</v>
       </c>
       <c r="L36" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M36" s="5"/>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A37" s="14">
+      <c r="A37" s="13">
         <v>1</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="D37" s="2"/>
       <c r="E37" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="F37" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="F37" s="2" t="s">
+      <c r="G37" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="H37" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="I37" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="I37" s="2" t="s">
-        <v>170</v>
-      </c>
       <c r="J37" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K37" s="5"/>
-      <c r="L37" s="5"/>
+      <c r="L37" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M37" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A38" s="14">
+      <c r="A38" s="13">
         <v>1</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D38" s="2"/>
       <c r="E38" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="F38" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="F38" s="2" t="s">
+      <c r="G38" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="G38" s="2" t="s">
+      <c r="H38" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="H38" s="2" t="s">
+      <c r="I38" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="I38" s="2" t="s">
-        <v>175</v>
-      </c>
       <c r="J38" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K38" s="5"/>
-      <c r="L38" s="5"/>
+      <c r="L38" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M38" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:13" ht="135" x14ac:dyDescent="0.25">
-      <c r="A39" s="14">
+      <c r="A39" s="13">
         <v>1</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
@@ -3430,124 +3493,128 @@
         <v>9</v>
       </c>
       <c r="L39" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M39" s="5"/>
     </row>
     <row r="40" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A40" s="14">
+      <c r="A40" s="13">
         <v>1</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="F40" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="G40" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G40" s="3" t="s">
+      <c r="H40" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="H40" s="3" t="s">
+      <c r="I40" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="I40" s="3" t="s">
-        <v>180</v>
-      </c>
       <c r="J40" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="K40" s="5"/>
-      <c r="L40" s="5"/>
+      <c r="L40" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M40" s="5"/>
     </row>
     <row r="41" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A41" s="14">
+      <c r="A41" s="13">
         <v>1</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F41" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="G41" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="G41" s="3" t="s">
+      <c r="H41" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="H41" s="3" t="s">
+      <c r="I41" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="I41" s="3" t="s">
-        <v>185</v>
-      </c>
       <c r="J41" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K41" s="5"/>
-      <c r="L41" s="5"/>
+      <c r="L41" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M41" s="5"/>
     </row>
     <row r="42" spans="1:13" ht="135" x14ac:dyDescent="0.25">
-      <c r="A42" s="14">
+      <c r="A42" s="13">
         <v>1</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="D42" s="2"/>
       <c r="E42" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="F42" s="3" t="s">
         <v>483</v>
       </c>
-      <c r="F42" s="3" t="s">
+      <c r="G42" s="3" t="s">
         <v>484</v>
       </c>
-      <c r="G42" s="3" t="s">
+      <c r="H42" s="3" t="s">
         <v>485</v>
       </c>
-      <c r="H42" s="3" t="s">
+      <c r="I42" s="3" t="s">
         <v>486</v>
       </c>
-      <c r="I42" s="3" t="s">
-        <v>487</v>
-      </c>
       <c r="J42" s="3" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="K42" s="5" t="s">
         <v>9</v>
       </c>
       <c r="L42" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M42" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:13" ht="135" x14ac:dyDescent="0.25">
-      <c r="A43" s="14">
+      <c r="A43" s="13">
         <v>1</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
@@ -3560,124 +3627,130 @@
         <v>9</v>
       </c>
       <c r="L43" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M43" s="5"/>
     </row>
     <row r="44" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A44" s="14">
+      <c r="A44" s="13">
         <v>1</v>
       </c>
       <c r="B44" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="D44" s="2"/>
       <c r="E44" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="F44" s="2" t="s">
+      <c r="G44" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="G44" s="2" t="s">
+      <c r="H44" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="H44" s="2" t="s">
+      <c r="I44" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="I44" s="2" t="s">
-        <v>190</v>
-      </c>
       <c r="J44" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K44" s="5"/>
-      <c r="L44" s="5"/>
+      <c r="L44" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M44" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A45" s="14">
+      <c r="A45" s="13">
         <v>1</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D45" s="2"/>
       <c r="E45" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="F45" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="F45" s="2" t="s">
+      <c r="G45" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="G45" s="2" t="s">
+      <c r="H45" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="H45" s="2" t="s">
+      <c r="I45" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="I45" s="2" t="s">
-        <v>195</v>
-      </c>
       <c r="J45" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="K45" s="5"/>
-      <c r="L45" s="5"/>
+      <c r="L45" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M45" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A46" s="14">
+      <c r="A46" s="13">
         <v>1</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D46" s="2"/>
       <c r="E46" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="F46" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="F46" s="2" t="s">
+      <c r="G46" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="H46" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="H46" s="2" t="s">
+      <c r="I46" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="I46" s="2" t="s">
-        <v>200</v>
-      </c>
       <c r="J46" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="K46" s="5"/>
-      <c r="L46" s="5"/>
+      <c r="L46" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M46" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:13" ht="75" x14ac:dyDescent="0.25">
-      <c r="A47" s="14">
+      <c r="A47" s="13">
         <v>1</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
@@ -3690,89 +3763,93 @@
         <v>9</v>
       </c>
       <c r="L47" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M47" s="5"/>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A48" s="14">
+      <c r="A48" s="13">
         <v>1</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="F48" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="F48" s="3" t="s">
+      <c r="G48" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="G48" s="3" t="s">
+      <c r="H48" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="H48" s="3" t="s">
+      <c r="I48" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="I48" s="3" t="s">
-        <v>205</v>
-      </c>
       <c r="J48" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K48" s="5"/>
-      <c r="L48" s="5"/>
+      <c r="L48" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M48" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A49" s="14">
+      <c r="A49" s="13">
         <v>1</v>
       </c>
       <c r="B49" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D49" s="2"/>
       <c r="E49" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="F49" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="F49" s="3" t="s">
+      <c r="G49" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="G49" s="3" t="s">
+      <c r="H49" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="H49" s="3" t="s">
+      <c r="I49" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="I49" s="3" t="s">
-        <v>210</v>
-      </c>
       <c r="J49" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K49" s="5"/>
-      <c r="L49" s="5"/>
+      <c r="L49" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M49" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:13" ht="270" x14ac:dyDescent="0.25">
-      <c r="A50" s="14">
+      <c r="A50" s="13">
         <v>1</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C50" s="12" t="s">
-        <v>503</v>
+      <c r="C50" s="11" t="s">
+        <v>502</v>
       </c>
       <c r="D50" s="2"/>
       <c r="E50" s="2"/>
@@ -3782,127 +3859,133 @@
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
       <c r="K50" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M50" s="5"/>
     </row>
     <row r="51" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="14">
+      <c r="A51" s="13">
         <v>1</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C51" s="12" t="s">
-        <v>437</v>
+      <c r="C51" s="11" t="s">
+        <v>436</v>
       </c>
       <c r="D51" s="2"/>
-      <c r="E51" s="12" t="s">
+      <c r="E51" s="11" t="s">
+        <v>342</v>
+      </c>
+      <c r="F51" s="11" t="s">
         <v>343</v>
       </c>
-      <c r="F51" s="12" t="s">
+      <c r="G51" s="11" t="s">
         <v>344</v>
       </c>
-      <c r="G51" s="12" t="s">
+      <c r="H51" s="11" t="s">
         <v>345</v>
       </c>
-      <c r="H51" s="12" t="s">
+      <c r="I51" s="11" t="s">
         <v>346</v>
       </c>
-      <c r="I51" s="12" t="s">
-        <v>347</v>
-      </c>
-      <c r="J51" s="12" t="s">
-        <v>343</v>
+      <c r="J51" s="11" t="s">
+        <v>342</v>
       </c>
       <c r="K51" s="5"/>
-      <c r="L51" s="5"/>
+      <c r="L51" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M51" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A52" s="14">
+      <c r="A52" s="13">
         <v>1</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C52" s="12" t="s">
-        <v>438</v>
+      <c r="C52" s="11" t="s">
+        <v>437</v>
       </c>
       <c r="D52" s="2"/>
-      <c r="E52" s="12" t="s">
+      <c r="E52" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="F52" s="11" t="s">
         <v>348</v>
       </c>
-      <c r="F52" s="12" t="s">
+      <c r="G52" s="11" t="s">
         <v>349</v>
       </c>
-      <c r="G52" s="12" t="s">
+      <c r="H52" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="H52" s="12" t="s">
+      <c r="I52" s="11" t="s">
         <v>351</v>
       </c>
-      <c r="I52" s="12" t="s">
-        <v>352</v>
-      </c>
-      <c r="J52" s="12" t="s">
-        <v>349</v>
+      <c r="J52" s="11" t="s">
+        <v>348</v>
       </c>
       <c r="K52" s="5"/>
-      <c r="L52" s="5"/>
+      <c r="L52" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M52" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A53" s="14">
+      <c r="A53" s="13">
         <v>1</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C53" s="12" t="s">
-        <v>439</v>
+      <c r="C53" s="11" t="s">
+        <v>438</v>
       </c>
       <c r="D53" s="2"/>
-      <c r="E53" s="12" t="s">
+      <c r="E53" s="11" t="s">
+        <v>352</v>
+      </c>
+      <c r="F53" s="11" t="s">
         <v>353</v>
       </c>
-      <c r="F53" s="12" t="s">
+      <c r="G53" s="11" t="s">
         <v>354</v>
       </c>
-      <c r="G53" s="12" t="s">
+      <c r="H53" s="11" t="s">
         <v>355</v>
       </c>
-      <c r="H53" s="12" t="s">
+      <c r="I53" s="11" t="s">
         <v>356</v>
       </c>
-      <c r="I53" s="12" t="s">
-        <v>357</v>
-      </c>
-      <c r="J53" s="12" t="s">
-        <v>357</v>
+      <c r="J53" s="11" t="s">
+        <v>356</v>
       </c>
       <c r="K53" s="5"/>
-      <c r="L53" s="5"/>
+      <c r="L53" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M53" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:13" ht="405" x14ac:dyDescent="0.25">
-      <c r="A54" s="14">
+      <c r="A54" s="13">
         <v>1</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C54" s="12" t="s">
-        <v>497</v>
+      <c r="C54" s="11" t="s">
+        <v>496</v>
       </c>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
@@ -3912,162 +3995,170 @@
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
       <c r="K54" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M54" s="5"/>
     </row>
     <row r="55" spans="1:13" ht="75" x14ac:dyDescent="0.25">
-      <c r="A55" s="14">
+      <c r="A55" s="13">
         <v>1</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C55" s="12" t="s">
-        <v>440</v>
+      <c r="C55" s="11" t="s">
+        <v>439</v>
       </c>
       <c r="D55" s="2"/>
-      <c r="E55" s="12" t="s">
+      <c r="E55" s="11" t="s">
+        <v>497</v>
+      </c>
+      <c r="F55" s="11" t="s">
         <v>498</v>
       </c>
-      <c r="F55" s="12" t="s">
+      <c r="G55" s="11" t="s">
         <v>499</v>
       </c>
-      <c r="G55" s="12" t="s">
+      <c r="H55" s="11" t="s">
         <v>500</v>
       </c>
-      <c r="H55" s="12" t="s">
+      <c r="I55" s="11" t="s">
         <v>501</v>
       </c>
-      <c r="I55" s="12" t="s">
-        <v>502</v>
-      </c>
-      <c r="J55" s="12" t="s">
-        <v>499</v>
+      <c r="J55" s="11" t="s">
+        <v>498</v>
       </c>
       <c r="K55" s="5"/>
-      <c r="L55" s="5"/>
+      <c r="L55" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M55" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A56" s="14">
+      <c r="A56" s="13">
         <v>1</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C56" s="12" t="s">
-        <v>442</v>
+      <c r="C56" s="11" t="s">
+        <v>441</v>
       </c>
       <c r="D56" s="2"/>
-      <c r="E56" s="12" t="s">
+      <c r="E56" s="11" t="s">
+        <v>357</v>
+      </c>
+      <c r="F56" s="11" t="s">
         <v>358</v>
       </c>
-      <c r="F56" s="12" t="s">
+      <c r="G56" s="11" t="s">
         <v>359</v>
       </c>
-      <c r="G56" s="12" t="s">
+      <c r="H56" s="11" t="s">
         <v>360</v>
       </c>
-      <c r="H56" s="12" t="s">
-        <v>361</v>
-      </c>
-      <c r="I56" s="12" t="s">
-        <v>348</v>
-      </c>
-      <c r="J56" s="12" t="s">
-        <v>359</v>
+      <c r="I56" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="J56" s="11" t="s">
+        <v>358</v>
       </c>
       <c r="K56" s="5"/>
-      <c r="L56" s="5"/>
+      <c r="L56" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M56" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A57" s="14">
+      <c r="A57" s="13">
         <v>1</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C57" s="12" t="s">
-        <v>443</v>
+      <c r="C57" s="11" t="s">
+        <v>442</v>
       </c>
       <c r="D57" s="2"/>
-      <c r="E57" s="12" t="s">
+      <c r="E57" s="11" t="s">
+        <v>361</v>
+      </c>
+      <c r="F57" s="11" t="s">
         <v>362</v>
       </c>
-      <c r="F57" s="12" t="s">
+      <c r="G57" s="11" t="s">
         <v>363</v>
       </c>
-      <c r="G57" s="12" t="s">
+      <c r="H57" s="11" t="s">
         <v>364</v>
       </c>
-      <c r="H57" s="12" t="s">
+      <c r="I57" s="11" t="s">
         <v>365</v>
       </c>
-      <c r="I57" s="12" t="s">
-        <v>366</v>
-      </c>
-      <c r="J57" s="12" t="s">
-        <v>366</v>
+      <c r="J57" s="11" t="s">
+        <v>365</v>
       </c>
       <c r="K57" s="5"/>
-      <c r="L57" s="5"/>
+      <c r="L57" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M57" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A58" s="14">
+      <c r="A58" s="13">
         <v>1</v>
       </c>
       <c r="B58" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C58" s="12" t="s">
-        <v>441</v>
+      <c r="C58" s="11" t="s">
+        <v>440</v>
       </c>
       <c r="D58" s="2"/>
-      <c r="E58" s="12" t="s">
+      <c r="E58" s="11" t="s">
+        <v>366</v>
+      </c>
+      <c r="F58" s="11" t="s">
         <v>367</v>
       </c>
-      <c r="F58" s="12" t="s">
+      <c r="G58" s="11" t="s">
         <v>368</v>
       </c>
-      <c r="G58" s="12" t="s">
+      <c r="H58" s="11" t="s">
         <v>369</v>
       </c>
-      <c r="H58" s="12" t="s">
+      <c r="I58" s="11" t="s">
         <v>370</v>
       </c>
-      <c r="I58" s="12" t="s">
-        <v>371</v>
-      </c>
-      <c r="J58" s="12" t="s">
-        <v>369</v>
+      <c r="J58" s="11" t="s">
+        <v>368</v>
       </c>
       <c r="K58" s="5"/>
-      <c r="L58" s="5"/>
+      <c r="L58" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M58" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:13" ht="165" x14ac:dyDescent="0.25">
-      <c r="A59" s="14">
+      <c r="A59" s="13">
         <v>1</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C59" s="12" t="s">
-        <v>496</v>
+      <c r="C59" s="11" t="s">
+        <v>495</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
@@ -4077,166 +4168,172 @@
       <c r="I59" s="2"/>
       <c r="J59" s="2"/>
       <c r="K59" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L59" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M59" s="5"/>
     </row>
     <row r="60" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A60" s="14">
+      <c r="A60" s="13">
         <v>1</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C60" s="12" t="s">
-        <v>444</v>
+      <c r="C60" s="11" t="s">
+        <v>443</v>
       </c>
       <c r="D60" s="2"/>
-      <c r="E60" s="12" t="s">
+      <c r="E60" s="11" t="s">
+        <v>371</v>
+      </c>
+      <c r="F60" s="11" t="s">
         <v>372</v>
       </c>
-      <c r="F60" s="12" t="s">
+      <c r="G60" s="11" t="s">
         <v>373</v>
       </c>
-      <c r="G60" s="12" t="s">
+      <c r="H60" s="11" t="s">
         <v>374</v>
       </c>
-      <c r="H60" s="12" t="s">
+      <c r="I60" s="11" t="s">
         <v>375</v>
       </c>
-      <c r="I60" s="12" t="s">
-        <v>376</v>
-      </c>
-      <c r="J60" s="12" t="s">
-        <v>373</v>
+      <c r="J60" s="11" t="s">
+        <v>372</v>
       </c>
       <c r="K60" s="5"/>
-      <c r="L60" s="5"/>
+      <c r="L60" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M60" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A61" s="14">
+      <c r="A61" s="13">
         <v>1</v>
       </c>
       <c r="B61" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C61" s="12" t="s">
-        <v>445</v>
+      <c r="C61" s="11" t="s">
+        <v>444</v>
       </c>
       <c r="D61" s="2"/>
-      <c r="E61" s="12" t="s">
+      <c r="E61" s="11" t="s">
+        <v>376</v>
+      </c>
+      <c r="F61" s="11" t="s">
         <v>377</v>
       </c>
-      <c r="F61" s="12" t="s">
+      <c r="G61" s="11" t="s">
         <v>378</v>
       </c>
-      <c r="G61" s="12" t="s">
+      <c r="H61" s="11" t="s">
         <v>379</v>
       </c>
-      <c r="H61" s="12" t="s">
+      <c r="I61" s="11" t="s">
         <v>380</v>
       </c>
-      <c r="I61" s="12" t="s">
-        <v>381</v>
-      </c>
-      <c r="J61" s="12" t="s">
-        <v>378</v>
+      <c r="J61" s="11" t="s">
+        <v>377</v>
       </c>
       <c r="K61" s="5"/>
-      <c r="L61" s="5"/>
+      <c r="L61" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M61" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A62" s="14">
+      <c r="A62" s="13">
         <v>1</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C62" s="12" t="s">
-        <v>446</v>
+      <c r="C62" s="11" t="s">
+        <v>445</v>
       </c>
       <c r="D62" s="2"/>
-      <c r="E62" s="12" t="s">
+      <c r="E62" s="11" t="s">
+        <v>381</v>
+      </c>
+      <c r="F62" s="11" t="s">
         <v>382</v>
       </c>
-      <c r="F62" s="12" t="s">
+      <c r="G62" s="11" t="s">
         <v>383</v>
       </c>
-      <c r="G62" s="12" t="s">
+      <c r="H62" s="11" t="s">
         <v>384</v>
       </c>
-      <c r="H62" s="12" t="s">
+      <c r="I62" s="11" t="s">
         <v>385</v>
       </c>
-      <c r="I62" s="12" t="s">
-        <v>386</v>
-      </c>
-      <c r="J62" s="12" t="s">
-        <v>382</v>
+      <c r="J62" s="11" t="s">
+        <v>381</v>
       </c>
       <c r="K62" s="5"/>
-      <c r="L62" s="5"/>
+      <c r="L62" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M62" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:13" ht="165" x14ac:dyDescent="0.25">
-      <c r="A63" s="14">
+      <c r="A63" s="13">
         <v>1</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C63" s="12" t="s">
-        <v>495</v>
+      <c r="C63" s="11" t="s">
+        <v>494</v>
       </c>
       <c r="D63" s="2"/>
-      <c r="E63" s="12" t="s">
+      <c r="E63" s="11" t="s">
+        <v>386</v>
+      </c>
+      <c r="F63" s="11" t="s">
         <v>387</v>
       </c>
-      <c r="F63" s="12" t="s">
+      <c r="G63" s="11" t="s">
         <v>388</v>
       </c>
-      <c r="G63" s="12" t="s">
+      <c r="H63" s="11" t="s">
         <v>389</v>
       </c>
-      <c r="H63" s="12" t="s">
+      <c r="I63" s="11" t="s">
         <v>390</v>
       </c>
-      <c r="I63" s="12" t="s">
-        <v>391</v>
-      </c>
-      <c r="J63" s="12" t="s">
-        <v>390</v>
+      <c r="J63" s="11" t="s">
+        <v>389</v>
       </c>
       <c r="K63" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L63" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M63" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:13" ht="255" x14ac:dyDescent="0.25">
-      <c r="A64" s="14">
+      <c r="A64" s="13">
         <v>1</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C64" s="12" t="s">
-        <v>494</v>
+      <c r="C64" s="11" t="s">
+        <v>493</v>
       </c>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
@@ -4246,92 +4343,96 @@
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
       <c r="K64" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L64" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M64" s="5"/>
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A65" s="14">
+      <c r="A65" s="13">
         <v>1</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C65" s="12" t="s">
-        <v>447</v>
+      <c r="C65" s="11" t="s">
+        <v>446</v>
       </c>
       <c r="D65" s="2"/>
-      <c r="E65" s="12" t="s">
+      <c r="E65" s="11" t="s">
+        <v>391</v>
+      </c>
+      <c r="F65" s="11" t="s">
         <v>392</v>
       </c>
-      <c r="F65" s="12" t="s">
+      <c r="G65" s="11" t="s">
         <v>393</v>
       </c>
-      <c r="G65" s="12" t="s">
+      <c r="H65" s="11" t="s">
         <v>394</v>
       </c>
-      <c r="H65" s="12" t="s">
+      <c r="I65" s="11" t="s">
         <v>395</v>
       </c>
-      <c r="I65" s="12" t="s">
-        <v>396</v>
-      </c>
-      <c r="J65" s="12" t="s">
-        <v>393</v>
+      <c r="J65" s="11" t="s">
+        <v>392</v>
       </c>
       <c r="K65" s="5"/>
-      <c r="L65" s="5"/>
+      <c r="L65" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M65" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A66" s="14">
+      <c r="A66" s="13">
         <v>1</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C66" s="12" t="s">
-        <v>448</v>
+      <c r="C66" s="11" t="s">
+        <v>447</v>
       </c>
       <c r="D66" s="2"/>
-      <c r="E66" s="12" t="s">
+      <c r="E66" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="F66" s="11" t="s">
         <v>397</v>
       </c>
-      <c r="F66" s="12" t="s">
+      <c r="G66" s="11" t="s">
         <v>398</v>
       </c>
-      <c r="G66" s="12" t="s">
+      <c r="H66" s="11" t="s">
         <v>399</v>
       </c>
-      <c r="H66" s="12" t="s">
+      <c r="I66" s="11" t="s">
         <v>400</v>
       </c>
-      <c r="I66" s="12" t="s">
-        <v>401</v>
-      </c>
-      <c r="J66" s="12" t="s">
-        <v>401</v>
+      <c r="J66" s="11" t="s">
+        <v>400</v>
       </c>
       <c r="K66" s="5"/>
-      <c r="L66" s="5"/>
+      <c r="L66" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M66" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:13" ht="105" x14ac:dyDescent="0.25">
-      <c r="A67" s="14">
+      <c r="A67" s="13">
         <v>1</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C67" s="12" t="s">
-        <v>493</v>
+      <c r="C67" s="11" t="s">
+        <v>492</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
@@ -4341,127 +4442,133 @@
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
       <c r="K67" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L67" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M67" s="5"/>
     </row>
     <row r="68" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A68" s="14">
+      <c r="A68" s="13">
         <v>1</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C68" s="12" t="s">
-        <v>449</v>
+      <c r="C68" s="11" t="s">
+        <v>448</v>
       </c>
       <c r="D68" s="2"/>
-      <c r="E68" s="12" t="s">
+      <c r="E68" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="F68" s="11" t="s">
         <v>402</v>
       </c>
-      <c r="F68" s="12" t="s">
+      <c r="G68" s="11" t="s">
         <v>403</v>
       </c>
-      <c r="G68" s="12" t="s">
+      <c r="H68" s="11" t="s">
         <v>404</v>
       </c>
-      <c r="H68" s="12" t="s">
+      <c r="I68" s="11" t="s">
         <v>405</v>
       </c>
-      <c r="I68" s="12" t="s">
-        <v>406</v>
-      </c>
-      <c r="J68" s="12" t="s">
-        <v>402</v>
+      <c r="J68" s="11" t="s">
+        <v>401</v>
       </c>
       <c r="K68" s="5"/>
-      <c r="L68" s="5"/>
+      <c r="L68" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M68" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A69" s="14">
+      <c r="A69" s="13">
         <v>1</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C69" s="12" t="s">
-        <v>450</v>
+      <c r="C69" s="11" t="s">
+        <v>449</v>
       </c>
       <c r="D69" s="2"/>
-      <c r="E69" s="12" t="s">
+      <c r="E69" s="11" t="s">
+        <v>406</v>
+      </c>
+      <c r="F69" s="11" t="s">
         <v>407</v>
       </c>
-      <c r="F69" s="12" t="s">
+      <c r="G69" s="11" t="s">
         <v>408</v>
       </c>
-      <c r="G69" s="12" t="s">
+      <c r="H69" s="11" t="s">
         <v>409</v>
       </c>
-      <c r="H69" s="12" t="s">
+      <c r="I69" s="11" t="s">
         <v>410</v>
       </c>
-      <c r="I69" s="12" t="s">
-        <v>411</v>
-      </c>
-      <c r="J69" s="12" t="s">
-        <v>409</v>
+      <c r="J69" s="11" t="s">
+        <v>408</v>
       </c>
       <c r="K69" s="5"/>
-      <c r="L69" s="5"/>
+      <c r="L69" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M69" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A70" s="14">
+      <c r="A70" s="13">
         <v>1</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C70" s="12" t="s">
-        <v>451</v>
+      <c r="C70" s="11" t="s">
+        <v>450</v>
       </c>
       <c r="D70" s="2"/>
-      <c r="E70" s="12" t="s">
+      <c r="E70" s="11" t="s">
+        <v>411</v>
+      </c>
+      <c r="F70" s="11" t="s">
         <v>412</v>
       </c>
-      <c r="F70" s="12" t="s">
+      <c r="G70" s="11" t="s">
         <v>413</v>
       </c>
-      <c r="G70" s="12" t="s">
+      <c r="H70" s="11" t="s">
         <v>414</v>
       </c>
-      <c r="H70" s="12" t="s">
+      <c r="I70" s="11" t="s">
         <v>415</v>
       </c>
-      <c r="I70" s="12" t="s">
-        <v>416</v>
-      </c>
-      <c r="J70" s="12" t="s">
-        <v>413</v>
+      <c r="J70" s="11" t="s">
+        <v>412</v>
       </c>
       <c r="K70" s="5"/>
-      <c r="L70" s="5"/>
+      <c r="L70" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M70" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="71" spans="1:13" ht="75" x14ac:dyDescent="0.25">
-      <c r="A71" s="14">
+      <c r="A71" s="13">
         <v>1</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C71" s="12" t="s">
-        <v>504</v>
+      <c r="C71" s="11" t="s">
+        <v>503</v>
       </c>
       <c r="D71" s="2"/>
       <c r="E71" s="2"/>
@@ -4471,92 +4578,96 @@
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
       <c r="K71" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L71" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M71" s="5"/>
     </row>
     <row r="72" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A72" s="14">
+      <c r="A72" s="13">
         <v>1</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C72" s="12" t="s">
-        <v>452</v>
+      <c r="C72" s="11" t="s">
+        <v>451</v>
       </c>
       <c r="D72" s="2"/>
-      <c r="E72" s="12" t="s">
+      <c r="E72" s="11" t="s">
+        <v>416</v>
+      </c>
+      <c r="F72" s="11" t="s">
         <v>417</v>
       </c>
-      <c r="F72" s="12" t="s">
+      <c r="G72" s="11" t="s">
         <v>418</v>
       </c>
-      <c r="G72" s="12" t="s">
+      <c r="H72" s="11" t="s">
         <v>419</v>
       </c>
-      <c r="H72" s="12" t="s">
+      <c r="I72" s="11" t="s">
         <v>420</v>
       </c>
-      <c r="I72" s="12" t="s">
-        <v>421</v>
-      </c>
-      <c r="J72" s="12" t="s">
-        <v>420</v>
+      <c r="J72" s="11" t="s">
+        <v>419</v>
       </c>
       <c r="K72" s="5"/>
-      <c r="L72" s="5"/>
+      <c r="L72" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M72" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="73" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A73" s="14">
+      <c r="A73" s="13">
         <v>1</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C73" s="12" t="s">
-        <v>453</v>
+      <c r="C73" s="11" t="s">
+        <v>452</v>
       </c>
       <c r="D73" s="2"/>
-      <c r="E73" s="12" t="s">
+      <c r="E73" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="F73" s="11" t="s">
         <v>422</v>
       </c>
-      <c r="F73" s="12" t="s">
+      <c r="G73" s="11" t="s">
         <v>423</v>
       </c>
-      <c r="G73" s="12" t="s">
+      <c r="H73" s="11" t="s">
         <v>424</v>
       </c>
-      <c r="H73" s="12" t="s">
+      <c r="I73" s="11" t="s">
         <v>425</v>
       </c>
-      <c r="I73" s="12" t="s">
-        <v>426</v>
-      </c>
-      <c r="J73" s="12" t="s">
-        <v>426</v>
+      <c r="J73" s="11" t="s">
+        <v>425</v>
       </c>
       <c r="K73" s="5"/>
-      <c r="L73" s="5"/>
+      <c r="L73" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M73" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="74" spans="1:13" ht="135" x14ac:dyDescent="0.25">
-      <c r="A74" s="14">
+      <c r="A74" s="13">
         <v>1</v>
       </c>
       <c r="B74" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C74" s="12" t="s">
-        <v>492</v>
+      <c r="C74" s="11" t="s">
+        <v>491</v>
       </c>
       <c r="D74" s="2"/>
       <c r="E74" s="2"/>
@@ -4566,92 +4677,96 @@
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
       <c r="K74" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L74" s="5" t="s">
-        <v>116</v>
+        <v>512</v>
       </c>
       <c r="M74" s="5"/>
     </row>
     <row r="75" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A75" s="14">
+      <c r="A75" s="13">
         <v>1</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C75" s="12" t="s">
-        <v>454</v>
+      <c r="C75" s="11" t="s">
+        <v>453</v>
       </c>
       <c r="D75" s="2"/>
-      <c r="E75" s="12" t="s">
+      <c r="E75" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="F75" s="11" t="s">
         <v>427</v>
       </c>
-      <c r="F75" s="12" t="s">
+      <c r="G75" s="11" t="s">
         <v>428</v>
       </c>
-      <c r="G75" s="12" t="s">
+      <c r="H75" s="11" t="s">
         <v>429</v>
       </c>
-      <c r="H75" s="12" t="s">
+      <c r="I75" s="11" t="s">
         <v>430</v>
       </c>
-      <c r="I75" s="12" t="s">
-        <v>431</v>
-      </c>
-      <c r="J75" s="12" t="s">
-        <v>427</v>
+      <c r="J75" s="11" t="s">
+        <v>426</v>
       </c>
       <c r="K75" s="5"/>
-      <c r="L75" s="5"/>
+      <c r="L75" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M75" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A76" s="14">
+      <c r="A76" s="13">
         <v>1</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C76" s="12" t="s">
-        <v>455</v>
+      <c r="C76" s="11" t="s">
+        <v>454</v>
       </c>
       <c r="D76" s="2"/>
-      <c r="E76" s="12" t="s">
+      <c r="E76" s="11" t="s">
+        <v>431</v>
+      </c>
+      <c r="F76" s="11" t="s">
         <v>432</v>
       </c>
-      <c r="F76" s="12" t="s">
+      <c r="G76" s="11" t="s">
         <v>433</v>
       </c>
-      <c r="G76" s="12" t="s">
+      <c r="H76" s="11" t="s">
         <v>434</v>
       </c>
-      <c r="H76" s="12" t="s">
+      <c r="I76" s="11" t="s">
         <v>435</v>
       </c>
-      <c r="I76" s="12" t="s">
-        <v>436</v>
-      </c>
-      <c r="J76" s="12" t="s">
-        <v>435</v>
+      <c r="J76" s="11" t="s">
+        <v>434</v>
       </c>
       <c r="K76" s="5"/>
-      <c r="L76" s="5"/>
+      <c r="L76" s="5" t="s">
+        <v>512</v>
+      </c>
       <c r="M76" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A77" s="14">
+      <c r="A77" s="13">
         <v>1</v>
       </c>
       <c r="B77" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D77" s="2"/>
       <c r="E77" s="3" t="s">
@@ -4672,25 +4787,25 @@
       <c r="J77" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="K77" s="11" t="s">
+      <c r="K77" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L77" s="10" t="s">
-        <v>116</v>
+      <c r="L77" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M77" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="78" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A78" s="14">
+      <c r="A78" s="13">
         <v>1</v>
       </c>
       <c r="B78" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D78" s="2"/>
       <c r="E78" s="3" t="s">
@@ -4711,25 +4826,25 @@
       <c r="J78" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="K78" s="11" t="s">
+      <c r="K78" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L78" s="10" t="s">
-        <v>116</v>
+      <c r="L78" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M78" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A79" s="14">
+      <c r="A79" s="13">
         <v>1</v>
       </c>
       <c r="B79" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="D79" s="2"/>
       <c r="E79" s="3" t="s">
@@ -4750,25 +4865,25 @@
       <c r="J79" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="K79" s="11" t="s">
+      <c r="K79" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L79" s="10" t="s">
-        <v>116</v>
+      <c r="L79" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M79" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A80" s="14">
+      <c r="A80" s="13">
         <v>1</v>
       </c>
       <c r="B80" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D80" s="2"/>
       <c r="E80" s="3" t="s">
@@ -4789,25 +4904,25 @@
       <c r="J80" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="K80" s="11" t="s">
+      <c r="K80" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L80" s="10" t="s">
-        <v>116</v>
+      <c r="L80" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M80" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A81" s="14">
+      <c r="A81" s="13">
         <v>1</v>
       </c>
       <c r="B81" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D81" s="2"/>
       <c r="E81" s="3" t="s">
@@ -4828,25 +4943,25 @@
       <c r="J81" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="K81" s="11" t="s">
+      <c r="K81" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L81" s="10" t="s">
-        <v>116</v>
+      <c r="L81" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M81" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="82" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A82" s="14">
+      <c r="A82" s="13">
         <v>1</v>
       </c>
       <c r="B82" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D82" s="2"/>
       <c r="E82" s="3" t="s">
@@ -4867,25 +4982,25 @@
       <c r="J82" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="K82" s="11" t="s">
+      <c r="K82" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L82" s="10" t="s">
-        <v>116</v>
+      <c r="L82" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M82" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="83" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A83" s="14">
+      <c r="A83" s="13">
         <v>1</v>
       </c>
       <c r="B83" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="D83" s="2"/>
       <c r="E83" s="3" t="s">
@@ -4906,25 +5021,25 @@
       <c r="J83" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="K83" s="11" t="s">
+      <c r="K83" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L83" s="10" t="s">
-        <v>116</v>
+      <c r="L83" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M83" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="84" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A84" s="14">
+      <c r="A84" s="13">
         <v>1</v>
       </c>
       <c r="B84" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D84" s="2"/>
       <c r="E84" s="3" t="s">
@@ -4945,25 +5060,25 @@
       <c r="J84" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="K84" s="11" t="s">
+      <c r="K84" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L84" s="10" t="s">
-        <v>116</v>
+      <c r="L84" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M84" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:13" ht="60" x14ac:dyDescent="0.25">
-      <c r="A85" s="14">
+      <c r="A85" s="13">
         <v>1</v>
       </c>
       <c r="B85" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="D85" s="2"/>
       <c r="E85" s="3" t="s">
@@ -4984,25 +5099,25 @@
       <c r="J85" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="K85" s="11" t="s">
+      <c r="K85" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L85" s="10" t="s">
-        <v>116</v>
+      <c r="L85" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M85" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="86" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A86" s="14">
+      <c r="A86" s="13">
         <v>1</v>
       </c>
       <c r="B86" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D86" s="2"/>
       <c r="E86" s="3" t="s">
@@ -5023,25 +5138,25 @@
       <c r="J86" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="K86" s="11" t="s">
+      <c r="K86" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L86" s="10" t="s">
-        <v>116</v>
+      <c r="L86" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M86" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="87" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A87" s="14">
+      <c r="A87" s="13">
         <v>1</v>
       </c>
       <c r="B87" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="D87" s="2"/>
       <c r="E87" s="3" t="s">
@@ -5062,25 +5177,25 @@
       <c r="J87" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="K87" s="11" t="s">
+      <c r="K87" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L87" s="10" t="s">
-        <v>116</v>
+      <c r="L87" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M87" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A88" s="14">
+      <c r="A88" s="13">
         <v>1</v>
       </c>
       <c r="B88" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D88" s="2"/>
       <c r="E88" s="3" t="s">
@@ -5101,25 +5216,25 @@
       <c r="J88" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="K88" s="11" t="s">
+      <c r="K88" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L88" s="10" t="s">
-        <v>116</v>
+      <c r="L88" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M88" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="89" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A89" s="14">
+      <c r="A89" s="13">
         <v>1</v>
       </c>
       <c r="B89" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="D89" s="2"/>
       <c r="E89" s="3" t="s">
@@ -5140,25 +5255,25 @@
       <c r="J89" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="K89" s="11" t="s">
+      <c r="K89" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L89" s="10" t="s">
-        <v>116</v>
+      <c r="L89" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M89" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="90" spans="1:13" ht="75" x14ac:dyDescent="0.25">
-      <c r="A90" s="14">
+      <c r="A90" s="13">
         <v>1</v>
       </c>
       <c r="B90" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D90" s="2"/>
       <c r="E90" s="3" t="s">
@@ -5179,25 +5294,25 @@
       <c r="J90" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="K90" s="11" t="s">
+      <c r="K90" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L90" s="10" t="s">
-        <v>116</v>
+      <c r="L90" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M90" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="91" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A91" s="14">
+      <c r="A91" s="13">
         <v>1</v>
       </c>
       <c r="B91" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="D91" s="2"/>
       <c r="E91" s="3" t="s">
@@ -5218,25 +5333,25 @@
       <c r="J91" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="K91" s="11" t="s">
+      <c r="K91" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L91" s="10" t="s">
-        <v>116</v>
+      <c r="L91" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M91" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="92" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A92" s="14">
+      <c r="A92" s="13">
         <v>1</v>
       </c>
       <c r="B92" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="D92" s="2"/>
       <c r="E92" s="3" t="s">
@@ -5257,25 +5372,25 @@
       <c r="J92" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="K92" s="11" t="s">
+      <c r="K92" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L92" s="10" t="s">
-        <v>116</v>
+      <c r="L92" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M92" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="93" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A93" s="14">
+      <c r="A93" s="13">
         <v>1</v>
       </c>
       <c r="B93" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="D93" s="2"/>
       <c r="E93" s="3" t="s">
@@ -5296,25 +5411,25 @@
       <c r="J93" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="K93" s="11" t="s">
+      <c r="K93" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L93" s="10" t="s">
-        <v>116</v>
+      <c r="L93" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M93" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="94" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A94" s="14">
+      <c r="A94" s="13">
         <v>1</v>
       </c>
       <c r="B94" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D94" s="2"/>
       <c r="E94" s="3" t="s">
@@ -5335,25 +5450,25 @@
       <c r="J94" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="K94" s="11" t="s">
+      <c r="K94" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L94" s="10" t="s">
-        <v>116</v>
+      <c r="L94" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M94" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="95" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A95" s="14">
+      <c r="A95" s="13">
         <v>1</v>
       </c>
       <c r="B95" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D95" s="2"/>
       <c r="E95" s="3" t="s">
@@ -5374,25 +5489,25 @@
       <c r="J95" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="K95" s="11" t="s">
+      <c r="K95" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L95" s="10" t="s">
-        <v>116</v>
+      <c r="L95" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M95" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="96" spans="1:13" ht="45" x14ac:dyDescent="0.25">
-      <c r="A96" s="14">
+      <c r="A96" s="13">
         <v>1</v>
       </c>
       <c r="B96" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D96" s="2"/>
       <c r="E96" s="3" t="s">
@@ -5413,11 +5528,11 @@
       <c r="J96" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="K96" s="11" t="s">
+      <c r="K96" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L96" s="10" t="s">
-        <v>116</v>
+      <c r="L96" s="5" t="s">
+        <v>512</v>
       </c>
       <c r="M96" s="6">
         <v>1</v>

</xml_diff>